<commit_message>
servo dumping pins were swapped, fixed.
</commit_message>
<xml_diff>
--- a/Car_Circuitry/Car_Circuitry_BOM.xlsx
+++ b/Car_Circuitry/Car_Circuitry_BOM.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Oasis\Documents\School\Assignments\Undergraduate Year 5\Chem-E Car Team\McMaster_Chem-E_Car_25-26\Car_Circuitry\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{72B925FD-C9F2-4550-AA5A-00320BBD05EA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{43BB5D52-D585-4A05-BF61-5680B2F02445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13620" xr2:uid="{EA864D17-A2FA-4459-BC44-DC5D03B4B2F6}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="22620" windowHeight="13620" xr2:uid="{57EE16C2-1588-46C7-AC60-D32C9E3DA668}"/>
   </bookViews>
   <sheets>
     <sheet name="Car_Circuitry_BOM" sheetId="1" r:id="rId1"/>
@@ -305,7 +305,7 @@
     <t>RCWE0805R100FKEA</t>
   </si>
   <si>
-    <t>390 Ω</t>
+    <t>400 Ω</t>
   </si>
   <si>
     <t>R2, R3</t>
@@ -353,7 +353,7 @@
     <t>ERA-6AEB204V</t>
   </si>
   <si>
-    <t>320 Ω</t>
+    <t>330 Ω</t>
   </si>
   <si>
     <t>R9</t>
@@ -818,7 +818,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{EB8C1EFA-50FD-475B-9A22-9E84E72D5A67}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DCEFBE8D-C481-435D-9AF0-F3D6748809DF}">
   <dimension ref="A1:F32"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>

</xml_diff>